<commit_message>
Updated Food Analysis file
</commit_message>
<xml_diff>
--- a/Excel Portfolio Projects/Food Price Analysis Project/Food Price Analysis Project.xlsx
+++ b/Excel Portfolio Projects/Food Price Analysis Project/Food Price Analysis Project.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a1ec44ccee5f08d5/Documents/Data Analysis/Portfolio/Excel Projects/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7393" documentId="8_{1A4C9D61-390D-4023-BEE6-CEA9014A7CC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{570634DC-3D13-481F-AF13-6B01C2164AFB}"/>
+  <xr:revisionPtr revIDLastSave="7400" documentId="8_{1A4C9D61-390D-4023-BEE6-CEA9014A7CC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B808222B-7CB7-47DA-A39C-2EB8FCB58ABC}"/>
   <bookViews>
     <workbookView xWindow="-38510" yWindow="-1790" windowWidth="38620" windowHeight="21100" activeTab="4" xr2:uid="{41A734D2-72BA-4562-B34B-238B193B17BA}"/>
   </bookViews>
@@ -24,7 +24,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="7" r:id="rId6"/>
+    <pivotCache cacheId="2" r:id="rId6"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
@@ -373,40 +373,6 @@
     <dxf>
       <font>
         <b/>
-        <i val="0"/>
-        <sz val="11"/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thick">
-          <color auto="1"/>
-        </left>
-        <right style="thick">
-          <color auto="1"/>
-        </right>
-        <top style="thick">
-          <color auto="1"/>
-        </top>
-        <bottom style="thick">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
         <color theme="1"/>
       </font>
       <fill>
@@ -448,6 +414,40 @@
       <font>
         <b/>
         <i val="0"/>
+        <sz val="11"/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7"/>
+        </patternFill>
+      </fill>
+      <border>
+        <left style="thick">
+          <color auto="1"/>
+        </left>
+        <right style="thick">
+          <color auto="1"/>
+        </right>
+        <top style="thick">
+          <color auto="1"/>
+        </top>
+        <bottom style="thick">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
       </font>
     </dxf>
   </dxfs>
@@ -456,12 +456,12 @@
       <tableStyleElement type="headerRow" dxfId="4"/>
     </tableStyle>
     <tableStyle name="Slicer Style 3" pivot="0" table="0" count="10" xr9:uid="{8962AC34-D094-41CA-8FE6-A0802A2C5389}">
+      <tableStyleElement type="wholeTable" dxfId="3"/>
+      <tableStyleElement type="headerRow" dxfId="2"/>
+    </tableStyle>
+    <tableStyle name="SlicerStyleDark2 2" pivot="0" table="0" count="10" xr9:uid="{BAE50467-7F35-40C7-A365-23CA1C12DB8D}">
       <tableStyleElement type="wholeTable" dxfId="1"/>
       <tableStyleElement type="headerRow" dxfId="0"/>
-    </tableStyle>
-    <tableStyle name="SlicerStyleDark2 2" pivot="0" table="0" count="10" xr9:uid="{BAE50467-7F35-40C7-A365-23CA1C12DB8D}">
-      <tableStyleElement type="wholeTable" dxfId="3"/>
-      <tableStyleElement type="headerRow" dxfId="2"/>
     </tableStyle>
   </tableStyles>
   <colors>
@@ -476,102 +476,6 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{46F421CA-312F-682f-3DD2-61675219B42D}">
       <x14:dxfs count="24">
-        <dxf>
-          <font>
-            <b/>
-            <i val="0"/>
-            <color theme="1"/>
-          </font>
-          <fill>
-            <patternFill>
-              <bgColor rgb="FFFFFF00"/>
-            </patternFill>
-          </fill>
-        </dxf>
-        <dxf>
-          <font>
-            <b/>
-            <i val="0"/>
-            <color theme="1"/>
-          </font>
-          <fill>
-            <patternFill>
-              <bgColor rgb="FFFFFF00"/>
-            </patternFill>
-          </fill>
-        </dxf>
-        <dxf>
-          <font>
-            <b/>
-            <i val="0"/>
-            <color theme="1"/>
-          </font>
-          <fill>
-            <patternFill>
-              <bgColor rgb="FFFFFF00"/>
-            </patternFill>
-          </fill>
-        </dxf>
-        <dxf>
-          <font>
-            <b/>
-            <i val="0"/>
-            <color theme="1"/>
-          </font>
-          <fill>
-            <patternFill>
-              <bgColor rgb="FFFFFF00"/>
-            </patternFill>
-          </fill>
-        </dxf>
-        <dxf>
-          <font>
-            <b/>
-            <i val="0"/>
-            <color theme="1"/>
-          </font>
-          <fill>
-            <patternFill>
-              <bgColor rgb="FFFFFF00"/>
-            </patternFill>
-          </fill>
-        </dxf>
-        <dxf>
-          <font>
-            <b/>
-            <i val="0"/>
-            <color theme="1"/>
-          </font>
-          <fill>
-            <patternFill>
-              <bgColor rgb="FFFFFF00"/>
-            </patternFill>
-          </fill>
-        </dxf>
-        <dxf>
-          <font>
-            <b/>
-            <i val="0"/>
-            <color theme="1"/>
-          </font>
-          <fill>
-            <patternFill>
-              <bgColor theme="7" tint="0.39994506668294322"/>
-            </patternFill>
-          </fill>
-        </dxf>
-        <dxf>
-          <font>
-            <b/>
-            <i val="0"/>
-            <color theme="1"/>
-          </font>
-          <fill>
-            <patternFill>
-              <bgColor theme="7" tint="0.39994506668294322"/>
-            </patternFill>
-          </fill>
-        </dxf>
         <dxf>
           <font>
             <color rgb="FF000000"/>
@@ -810,6 +714,102 @@
         </dxf>
         <dxf>
           <font>
+            <b/>
+            <i val="0"/>
+            <color theme="1"/>
+          </font>
+          <fill>
+            <patternFill>
+              <bgColor rgb="FFFFFF00"/>
+            </patternFill>
+          </fill>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <color theme="1"/>
+          </font>
+          <fill>
+            <patternFill>
+              <bgColor rgb="FFFFFF00"/>
+            </patternFill>
+          </fill>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <color theme="1"/>
+          </font>
+          <fill>
+            <patternFill>
+              <bgColor rgb="FFFFFF00"/>
+            </patternFill>
+          </fill>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <color theme="1"/>
+          </font>
+          <fill>
+            <patternFill>
+              <bgColor rgb="FFFFFF00"/>
+            </patternFill>
+          </fill>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <color theme="1"/>
+          </font>
+          <fill>
+            <patternFill>
+              <bgColor rgb="FFFFFF00"/>
+            </patternFill>
+          </fill>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <color theme="1"/>
+          </font>
+          <fill>
+            <patternFill>
+              <bgColor rgb="FFFFFF00"/>
+            </patternFill>
+          </fill>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <color theme="1"/>
+          </font>
+          <fill>
+            <patternFill>
+              <bgColor theme="7" tint="0.39994506668294322"/>
+            </patternFill>
+          </fill>
+        </dxf>
+        <dxf>
+          <font>
+            <b/>
+            <i val="0"/>
+            <color theme="1"/>
+          </font>
+          <fill>
+            <patternFill>
+              <bgColor theme="7" tint="0.39994506668294322"/>
+            </patternFill>
+          </fill>
+        </dxf>
+        <dxf>
+          <font>
             <color theme="0"/>
           </font>
           <fill>
@@ -906,6 +906,18 @@
         </x14:slicerStyle>
         <x14:slicerStyle name="Slicer Style 3">
           <x14:slicerStyleElements>
+            <x14:slicerStyleElement type="unselectedItemWithData" dxfId="15"/>
+            <x14:slicerStyleElement type="unselectedItemWithNoData" dxfId="14"/>
+            <x14:slicerStyleElement type="selectedItemWithData" dxfId="13"/>
+            <x14:slicerStyleElement type="selectedItemWithNoData" dxfId="12"/>
+            <x14:slicerStyleElement type="hoveredUnselectedItemWithData" dxfId="11"/>
+            <x14:slicerStyleElement type="hoveredSelectedItemWithData" dxfId="10"/>
+            <x14:slicerStyleElement type="hoveredUnselectedItemWithNoData" dxfId="9"/>
+            <x14:slicerStyleElement type="hoveredSelectedItemWithNoData" dxfId="8"/>
+          </x14:slicerStyleElements>
+        </x14:slicerStyle>
+        <x14:slicerStyle name="SlicerStyleDark2 2">
+          <x14:slicerStyleElements>
             <x14:slicerStyleElement type="unselectedItemWithData" dxfId="7"/>
             <x14:slicerStyleElement type="unselectedItemWithNoData" dxfId="6"/>
             <x14:slicerStyleElement type="selectedItemWithData" dxfId="5"/>
@@ -914,18 +926,6 @@
             <x14:slicerStyleElement type="hoveredSelectedItemWithData" dxfId="2"/>
             <x14:slicerStyleElement type="hoveredUnselectedItemWithNoData" dxfId="1"/>
             <x14:slicerStyleElement type="hoveredSelectedItemWithNoData" dxfId="0"/>
-          </x14:slicerStyleElements>
-        </x14:slicerStyle>
-        <x14:slicerStyle name="SlicerStyleDark2 2">
-          <x14:slicerStyleElements>
-            <x14:slicerStyleElement type="unselectedItemWithData" dxfId="15"/>
-            <x14:slicerStyleElement type="unselectedItemWithNoData" dxfId="14"/>
-            <x14:slicerStyleElement type="selectedItemWithData" dxfId="13"/>
-            <x14:slicerStyleElement type="selectedItemWithNoData" dxfId="12"/>
-            <x14:slicerStyleElement type="hoveredUnselectedItemWithData" dxfId="11"/>
-            <x14:slicerStyleElement type="hoveredSelectedItemWithData" dxfId="10"/>
-            <x14:slicerStyleElement type="hoveredUnselectedItemWithNoData" dxfId="9"/>
-            <x14:slicerStyleElement type="hoveredSelectedItemWithNoData" dxfId="8"/>
           </x14:slicerStyleElements>
         </x14:slicerStyle>
       </x14:slicerStyles>
@@ -1147,7 +1147,7 @@
             <a:effectLst/>
           </c:spPr>
           <c:txPr>
-            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" wrap="square" anchor="ctr" anchorCtr="1"/>
             <a:lstStyle/>
             <a:p>
               <a:pPr>
@@ -1621,7 +1621,7 @@
               <a:effectLst/>
             </c:spPr>
             <c:txPr>
-              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" wrap="square" anchor="ctr" anchorCtr="1"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
@@ -2199,7 +2199,7 @@
             <a:effectLst/>
           </c:spPr>
           <c:txPr>
-            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" wrap="square" anchor="ctr" anchorCtr="1"/>
             <a:lstStyle/>
             <a:p>
               <a:pPr>
@@ -2663,7 +2663,7 @@
               <a:effectLst/>
             </c:spPr>
             <c:txPr>
-              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" wrap="square" anchor="ctr" anchorCtr="1"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
@@ -3148,6 +3148,15 @@
               <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
+          <c:showLegendKey val="1"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="1"/>
+          <c:showSerName val="1"/>
+          <c:showPercent val="1"/>
+          <c:showBubbleSize val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
         </c:dLbl>
       </c:pivotFmt>
       <c:pivotFmt>
@@ -3192,6 +3201,15 @@
               <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
+          <c:showLegendKey val="1"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="1"/>
+          <c:showSerName val="1"/>
+          <c:showPercent val="1"/>
+          <c:showBubbleSize val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
         </c:dLbl>
       </c:pivotFmt>
       <c:pivotFmt>
@@ -3218,7 +3236,7 @@
             <a:effectLst/>
           </c:spPr>
           <c:txPr>
-            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" wrap="square" anchor="ctr" anchorCtr="1"/>
             <a:lstStyle/>
             <a:p>
               <a:pPr>
@@ -3682,7 +3700,7 @@
               <a:effectLst/>
             </c:spPr>
             <c:txPr>
-              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" wrap="square" anchor="ctr" anchorCtr="1"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
@@ -4261,7 +4279,7 @@
             <a:effectLst/>
           </c:spPr>
           <c:txPr>
-            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" wrap="square" anchor="ctr" anchorCtr="1"/>
             <a:lstStyle/>
             <a:p>
               <a:pPr>
@@ -4725,7 +4743,7 @@
               <a:effectLst/>
             </c:spPr>
             <c:txPr>
-              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" wrap="square" anchor="ctr" anchorCtr="1"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
@@ -5306,7 +5324,7 @@
             <a:effectLst/>
           </c:spPr>
           <c:txPr>
-            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" wrap="square" anchor="ctr" anchorCtr="1"/>
             <a:lstStyle/>
             <a:p>
               <a:pPr>
@@ -5770,7 +5788,7 @@
               <a:effectLst/>
             </c:spPr>
             <c:txPr>
-              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" wrap="square" anchor="ctr" anchorCtr="1"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
@@ -12533,15 +12551,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>406400</xdr:colOff>
+      <xdr:colOff>409575</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>180975</xdr:rowOff>
+      <xdr:rowOff>184150</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
       <xdr:colOff>304799</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>165099</xdr:rowOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -12617,7 +12635,7 @@
       <xdr:col>28</xdr:col>
       <xdr:colOff>171450</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>139700</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -12766,15 +12784,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>21</xdr:col>
-      <xdr:colOff>390525</xdr:colOff>
+      <xdr:colOff>393701</xdr:colOff>
       <xdr:row>15</xdr:row>
       <xdr:rowOff>41272</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>37</xdr:col>
-      <xdr:colOff>593725</xdr:colOff>
+      <xdr:colOff>527051</xdr:colOff>
       <xdr:row>30</xdr:row>
-      <xdr:rowOff>31750</xdr:rowOff>
+      <xdr:rowOff>34925</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -12789,8 +12807,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13192125" y="2898772"/>
-          <a:ext cx="9956800" cy="2847978"/>
+          <a:off x="13195301" y="2898772"/>
+          <a:ext cx="9886950" cy="2851153"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -13796,10 +13814,10 @@
       <xdr:rowOff>187324</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>38</xdr:col>
-      <xdr:colOff>34925</xdr:colOff>
+      <xdr:col>37</xdr:col>
+      <xdr:colOff>527050</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>107950</xdr:rowOff>
+      <xdr:rowOff>111125</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -13815,7 +13833,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="13217525" y="187324"/>
-          <a:ext cx="9982200" cy="2587626"/>
+          <a:ext cx="9864725" cy="2590801"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -13964,18 +13982,15 @@
             </a:rPr>
             <a:t> Target.</a:t>
           </a:r>
-          <a:r>
-            <a:rPr lang="en-GB" sz="1050" b="1" i="1">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>.</a:t>
-          </a:r>
+          <a:endParaRPr lang="en-GB" sz="1050" b="1" i="1">
+            <a:solidFill>
+              <a:schemeClr val="dk1"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+          </a:endParaRPr>
         </a:p>
         <a:p>
           <a:r>
@@ -14516,7 +14531,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>288924</xdr:colOff>
+      <xdr:colOff>152400</xdr:colOff>
       <xdr:row>43</xdr:row>
       <xdr:rowOff>19050</xdr:rowOff>
     </xdr:to>
@@ -14534,7 +14549,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="365124" y="5654676"/>
-          <a:ext cx="10287000" cy="2555874"/>
+          <a:ext cx="10150476" cy="2555874"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -14842,13 +14857,13 @@
       <xdr:col>21</xdr:col>
       <xdr:colOff>396876</xdr:colOff>
       <xdr:row>30</xdr:row>
-      <xdr:rowOff>184150</xdr:rowOff>
+      <xdr:rowOff>187325</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>37</xdr:col>
-      <xdr:colOff>473076</xdr:colOff>
+      <xdr:colOff>565150</xdr:colOff>
       <xdr:row>43</xdr:row>
-      <xdr:rowOff>31751</xdr:rowOff>
+      <xdr:rowOff>34926</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -14863,8 +14878,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13198476" y="5899150"/>
-          <a:ext cx="9829800" cy="2324101"/>
+          <a:off x="13198476" y="5902325"/>
+          <a:ext cx="9921874" cy="2324101"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -16068,376 +16083,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{6A95122E-CF41-4DA1-B1E7-134442D916EB}" name="PivotTable8" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="11">
-  <location ref="L8:M27" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="6">
-    <pivotField axis="axisRow" showAll="0">
-      <items count="4">
-        <item x="1"/>
-        <item x="2"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="6">
-        <item x="2"/>
-        <item x="3"/>
-        <item x="1"/>
-        <item x="4"/>
-        <item x="0"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField dataField="1" numFmtId="164" showAll="0"/>
-    <pivotField numFmtId="14" showAll="0">
-      <items count="5">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0" defaultSubtotal="0"/>
-    <pivotField showAll="0" defaultSubtotal="0">
-      <items count="14">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item x="11"/>
-        <item x="12"/>
-        <item x="13"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="2">
-    <field x="0"/>
-    <field x="1"/>
-  </rowFields>
-  <rowItems count="19">
-    <i>
-      <x/>
-    </i>
-    <i r="1">
-      <x/>
-    </i>
-    <i r="1">
-      <x v="1"/>
-    </i>
-    <i r="1">
-      <x v="2"/>
-    </i>
-    <i r="1">
-      <x v="3"/>
-    </i>
-    <i r="1">
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i r="1">
-      <x/>
-    </i>
-    <i r="1">
-      <x v="1"/>
-    </i>
-    <i r="1">
-      <x v="2"/>
-    </i>
-    <i r="1">
-      <x v="3"/>
-    </i>
-    <i r="1">
-      <x v="4"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i r="1">
-      <x/>
-    </i>
-    <i r="1">
-      <x v="1"/>
-    </i>
-    <i r="1">
-      <x v="2"/>
-    </i>
-    <i r="1">
-      <x v="3"/>
-    </i>
-    <i r="1">
-      <x v="4"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Max of Price" fld="2" subtotal="max" baseField="0" baseItem="0" numFmtId="164"/>
-  </dataFields>
-  <chartFormats count="16">
-    <chartFormat chart="3" format="12" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="3" format="13">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="3">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-          <reference field="1" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="3" format="14">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="3">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-          <reference field="1" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="3" format="15">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="3">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-          <reference field="1" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="3" format="16">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="3">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-          <reference field="1" count="1" selected="0">
-            <x v="3"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="3" format="17">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="3">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-          <reference field="1" count="1" selected="0">
-            <x v="4"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="3" format="18">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="3">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-          <reference field="1" count="1" selected="0">
-            <x v="4"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="3" format="19">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="3">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-          <reference field="1" count="1" selected="0">
-            <x v="3"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="3" format="20">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="3">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-          <reference field="1" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="3" format="21">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="3">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-          <reference field="1" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="3" format="22">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="3">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-          <reference field="1" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="3" format="23">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="3">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="1" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="3" format="24">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="3">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="1" count="1" selected="0">
-            <x v="4"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="3" format="25">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="3">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="1" count="1" selected="0">
-            <x v="3"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="3" format="26">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="3">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="1" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="3" format="27">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="3">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="0" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="1" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9DD450E6-C956-49DC-91E4-82267813AE3A}" name="PivotTable5" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9DD450E6-C956-49DC-91E4-82267813AE3A}" name="PivotTable5" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6">
   <location ref="I29:J46" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="6">
     <pivotField axis="axisRow" showAll="0">
@@ -17220,8 +16866,745 @@
 </pivotTableDefinition>
 </file>
 
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{7559EBD1-7AE6-457F-AF35-5A2E887508ED}" name="PivotTable3" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
+  <location ref="F29:G46" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="6">
+    <pivotField axis="axisRow" showAll="0">
+      <items count="4">
+        <item x="1"/>
+        <item x="2"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="6">
+        <item h="1" x="2"/>
+        <item x="3"/>
+        <item h="1" x="1"/>
+        <item h="1" x="4"/>
+        <item h="1" x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" numFmtId="164" showAll="0"/>
+    <pivotField numFmtId="14" showAll="0">
+      <items count="5">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="369">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item x="15"/>
+        <item x="16"/>
+        <item x="17"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item x="20"/>
+        <item x="21"/>
+        <item x="22"/>
+        <item x="23"/>
+        <item x="24"/>
+        <item x="25"/>
+        <item x="26"/>
+        <item x="27"/>
+        <item x="28"/>
+        <item x="29"/>
+        <item x="30"/>
+        <item x="31"/>
+        <item x="32"/>
+        <item x="33"/>
+        <item x="34"/>
+        <item x="35"/>
+        <item x="36"/>
+        <item x="37"/>
+        <item x="38"/>
+        <item x="39"/>
+        <item x="40"/>
+        <item x="41"/>
+        <item x="42"/>
+        <item x="43"/>
+        <item x="44"/>
+        <item x="45"/>
+        <item x="46"/>
+        <item x="47"/>
+        <item x="48"/>
+        <item x="49"/>
+        <item x="50"/>
+        <item x="51"/>
+        <item x="52"/>
+        <item x="53"/>
+        <item x="54"/>
+        <item x="55"/>
+        <item x="56"/>
+        <item x="57"/>
+        <item x="58"/>
+        <item x="59"/>
+        <item x="60"/>
+        <item x="61"/>
+        <item x="62"/>
+        <item x="63"/>
+        <item x="64"/>
+        <item x="65"/>
+        <item x="66"/>
+        <item x="67"/>
+        <item x="68"/>
+        <item x="69"/>
+        <item x="70"/>
+        <item x="71"/>
+        <item x="72"/>
+        <item x="73"/>
+        <item x="74"/>
+        <item x="75"/>
+        <item x="76"/>
+        <item x="77"/>
+        <item x="78"/>
+        <item x="79"/>
+        <item x="80"/>
+        <item x="81"/>
+        <item x="82"/>
+        <item x="83"/>
+        <item x="84"/>
+        <item x="85"/>
+        <item x="86"/>
+        <item x="87"/>
+        <item x="88"/>
+        <item x="89"/>
+        <item x="90"/>
+        <item x="91"/>
+        <item x="92"/>
+        <item x="93"/>
+        <item x="94"/>
+        <item x="95"/>
+        <item x="96"/>
+        <item x="97"/>
+        <item x="98"/>
+        <item x="99"/>
+        <item x="100"/>
+        <item x="101"/>
+        <item x="102"/>
+        <item x="103"/>
+        <item x="104"/>
+        <item x="105"/>
+        <item x="106"/>
+        <item x="107"/>
+        <item x="108"/>
+        <item x="109"/>
+        <item x="110"/>
+        <item x="111"/>
+        <item x="112"/>
+        <item x="113"/>
+        <item x="114"/>
+        <item x="115"/>
+        <item x="116"/>
+        <item x="117"/>
+        <item x="118"/>
+        <item x="119"/>
+        <item x="120"/>
+        <item x="121"/>
+        <item x="122"/>
+        <item x="123"/>
+        <item x="124"/>
+        <item x="125"/>
+        <item x="126"/>
+        <item x="127"/>
+        <item x="128"/>
+        <item x="129"/>
+        <item x="130"/>
+        <item x="131"/>
+        <item x="132"/>
+        <item x="133"/>
+        <item x="134"/>
+        <item x="135"/>
+        <item x="136"/>
+        <item x="137"/>
+        <item x="138"/>
+        <item x="139"/>
+        <item x="140"/>
+        <item x="141"/>
+        <item x="142"/>
+        <item x="143"/>
+        <item x="144"/>
+        <item x="145"/>
+        <item x="146"/>
+        <item x="147"/>
+        <item x="148"/>
+        <item x="149"/>
+        <item x="150"/>
+        <item x="151"/>
+        <item x="152"/>
+        <item x="153"/>
+        <item x="154"/>
+        <item x="155"/>
+        <item x="156"/>
+        <item x="157"/>
+        <item x="158"/>
+        <item x="159"/>
+        <item x="160"/>
+        <item x="161"/>
+        <item x="162"/>
+        <item x="163"/>
+        <item x="164"/>
+        <item x="165"/>
+        <item x="166"/>
+        <item x="167"/>
+        <item x="168"/>
+        <item x="169"/>
+        <item x="170"/>
+        <item x="171"/>
+        <item x="172"/>
+        <item x="173"/>
+        <item x="174"/>
+        <item x="175"/>
+        <item x="176"/>
+        <item x="177"/>
+        <item x="178"/>
+        <item x="179"/>
+        <item x="180"/>
+        <item x="181"/>
+        <item x="182"/>
+        <item x="183"/>
+        <item x="184"/>
+        <item x="185"/>
+        <item x="186"/>
+        <item x="187"/>
+        <item x="188"/>
+        <item x="189"/>
+        <item x="190"/>
+        <item x="191"/>
+        <item x="192"/>
+        <item x="193"/>
+        <item x="194"/>
+        <item x="195"/>
+        <item x="196"/>
+        <item x="197"/>
+        <item x="198"/>
+        <item x="199"/>
+        <item x="200"/>
+        <item x="201"/>
+        <item x="202"/>
+        <item x="203"/>
+        <item x="204"/>
+        <item x="205"/>
+        <item x="206"/>
+        <item x="207"/>
+        <item x="208"/>
+        <item x="209"/>
+        <item x="210"/>
+        <item x="211"/>
+        <item x="212"/>
+        <item x="213"/>
+        <item x="214"/>
+        <item x="215"/>
+        <item x="216"/>
+        <item x="217"/>
+        <item x="218"/>
+        <item x="219"/>
+        <item x="220"/>
+        <item x="221"/>
+        <item x="222"/>
+        <item x="223"/>
+        <item x="224"/>
+        <item x="225"/>
+        <item x="226"/>
+        <item x="227"/>
+        <item x="228"/>
+        <item x="229"/>
+        <item x="230"/>
+        <item x="231"/>
+        <item x="232"/>
+        <item x="233"/>
+        <item x="234"/>
+        <item x="235"/>
+        <item x="236"/>
+        <item x="237"/>
+        <item x="238"/>
+        <item x="239"/>
+        <item x="240"/>
+        <item x="241"/>
+        <item x="242"/>
+        <item x="243"/>
+        <item x="244"/>
+        <item x="245"/>
+        <item x="246"/>
+        <item x="247"/>
+        <item x="248"/>
+        <item x="249"/>
+        <item x="250"/>
+        <item x="251"/>
+        <item x="252"/>
+        <item x="253"/>
+        <item x="254"/>
+        <item x="255"/>
+        <item x="256"/>
+        <item x="257"/>
+        <item x="258"/>
+        <item x="259"/>
+        <item x="260"/>
+        <item x="261"/>
+        <item x="262"/>
+        <item x="263"/>
+        <item x="264"/>
+        <item x="265"/>
+        <item x="266"/>
+        <item x="267"/>
+        <item x="268"/>
+        <item x="269"/>
+        <item x="270"/>
+        <item x="271"/>
+        <item x="272"/>
+        <item x="273"/>
+        <item x="274"/>
+        <item x="275"/>
+        <item x="276"/>
+        <item x="277"/>
+        <item x="278"/>
+        <item x="279"/>
+        <item x="280"/>
+        <item x="281"/>
+        <item x="282"/>
+        <item x="283"/>
+        <item x="284"/>
+        <item x="285"/>
+        <item x="286"/>
+        <item x="287"/>
+        <item x="288"/>
+        <item x="289"/>
+        <item x="290"/>
+        <item x="291"/>
+        <item x="292"/>
+        <item x="293"/>
+        <item x="294"/>
+        <item x="295"/>
+        <item x="296"/>
+        <item x="297"/>
+        <item x="298"/>
+        <item x="299"/>
+        <item x="300"/>
+        <item x="301"/>
+        <item x="302"/>
+        <item x="303"/>
+        <item x="304"/>
+        <item x="305"/>
+        <item x="306"/>
+        <item x="307"/>
+        <item x="308"/>
+        <item x="309"/>
+        <item x="310"/>
+        <item x="311"/>
+        <item x="312"/>
+        <item x="313"/>
+        <item x="314"/>
+        <item x="315"/>
+        <item x="316"/>
+        <item x="317"/>
+        <item x="318"/>
+        <item x="319"/>
+        <item x="320"/>
+        <item x="321"/>
+        <item x="322"/>
+        <item x="323"/>
+        <item x="324"/>
+        <item x="325"/>
+        <item x="326"/>
+        <item x="327"/>
+        <item x="328"/>
+        <item x="329"/>
+        <item x="330"/>
+        <item x="331"/>
+        <item x="332"/>
+        <item x="333"/>
+        <item x="334"/>
+        <item x="335"/>
+        <item x="336"/>
+        <item x="337"/>
+        <item x="338"/>
+        <item x="339"/>
+        <item x="340"/>
+        <item x="341"/>
+        <item x="342"/>
+        <item x="343"/>
+        <item x="344"/>
+        <item x="345"/>
+        <item x="346"/>
+        <item x="347"/>
+        <item x="348"/>
+        <item x="349"/>
+        <item x="350"/>
+        <item x="351"/>
+        <item x="352"/>
+        <item x="353"/>
+        <item x="354"/>
+        <item x="355"/>
+        <item x="356"/>
+        <item x="357"/>
+        <item x="358"/>
+        <item x="359"/>
+        <item x="360"/>
+        <item x="361"/>
+        <item x="362"/>
+        <item x="363"/>
+        <item x="364"/>
+        <item x="365"/>
+        <item x="366"/>
+        <item x="367"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="15">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="3">
+    <field x="1"/>
+    <field x="0"/>
+    <field x="5"/>
+  </rowFields>
+  <rowItems count="17">
+    <i>
+      <x v="1"/>
+    </i>
+    <i r="1">
+      <x/>
+    </i>
+    <i r="2">
+      <x v="1"/>
+    </i>
+    <i r="2">
+      <x v="2"/>
+    </i>
+    <i r="2">
+      <x v="3"/>
+    </i>
+    <i r="2">
+      <x v="4"/>
+    </i>
+    <i r="1">
+      <x v="1"/>
+    </i>
+    <i r="2">
+      <x v="1"/>
+    </i>
+    <i r="2">
+      <x v="2"/>
+    </i>
+    <i r="2">
+      <x v="3"/>
+    </i>
+    <i r="2">
+      <x v="4"/>
+    </i>
+    <i r="1">
+      <x v="2"/>
+    </i>
+    <i r="2">
+      <x v="1"/>
+    </i>
+    <i r="2">
+      <x v="2"/>
+    </i>
+    <i r="2">
+      <x v="3"/>
+    </i>
+    <i r="2">
+      <x v="4"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of Price" fld="2" baseField="0" baseItem="0" numFmtId="164"/>
+  </dataFields>
+  <chartFormats count="14">
+    <chartFormat chart="2" format="0" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="4" format="2" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="4" format="3">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="4">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+          <reference field="5" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="4" format="4">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="4">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+          <reference field="5" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="4" format="5">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="4">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+          <reference field="5" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="4" format="6">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="4">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+          <reference field="5" count="1" selected="0">
+            <x v="4"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="4" format="7">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="4">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+          <reference field="5" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="4" format="8">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="4">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+          <reference field="5" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="4" format="9">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="4">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+          <reference field="5" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="4" format="10">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="4">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+          <reference field="5" count="1" selected="0">
+            <x v="4"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="4" format="11">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="4">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+          <reference field="5" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="4" format="12">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="4">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+          <reference field="5" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="4" format="13">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="4">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+          <reference field="5" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="4" format="14">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="4">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+          <reference field="5" count="1" selected="0">
+            <x v="4"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{48790682-40B4-417D-80F3-F9CC7331BF70}" name="PivotTable4" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{48790682-40B4-417D-80F3-F9CC7331BF70}" name="PivotTable4" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="4">
   <location ref="I10:J27" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="6">
     <pivotField axis="axisRow" showAll="0">
@@ -17958,7 +18341,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0DDFB93E-C9AF-47D3-B545-E3855D408557}" name="PivotTable2" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{0DDFB93E-C9AF-47D3-B545-E3855D408557}" name="PivotTable2" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10">
   <location ref="F10:G27" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="6">
     <pivotField axis="axisRow" showAll="0">
@@ -18695,7 +19078,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A0F3CF21-2C0C-4840-B45F-C6576F11A36B}" name="PivotTable1" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A0F3CF21-2C0C-4840-B45F-C6576F11A36B}" name="PivotTable1" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="F2:G8" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="6">
     <pivotField showAll="0">
@@ -19161,7 +19544,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{79AB6943-C741-4C62-87C8-B0580BBDAEEF}" name="PivotTable6" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{79AB6943-C741-4C62-87C8-B0580BBDAEEF}" name="PivotTable6" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10">
   <location ref="L29:M46" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="6">
     <pivotField axis="axisRow" showAll="0">
@@ -19898,8 +20281,8 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{7559EBD1-7AE6-457F-AF35-5A2E887508ED}" name="PivotTable3" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="5">
-  <location ref="F29:G46" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{6A95122E-CF41-4DA1-B1E7-134442D916EB}" name="PivotTable8" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="11">
+  <location ref="L8:M27" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="6">
     <pivotField axis="axisRow" showAll="0">
       <items count="4">
@@ -19911,11 +20294,11 @@
     </pivotField>
     <pivotField axis="axisRow" showAll="0">
       <items count="6">
-        <item h="1" x="2"/>
+        <item x="2"/>
         <item x="3"/>
-        <item h="1" x="1"/>
-        <item h="1" x="4"/>
-        <item h="1" x="0"/>
+        <item x="1"/>
+        <item x="4"/>
+        <item x="0"/>
         <item t="default"/>
       </items>
     </pivotField>
@@ -19929,8 +20312,9 @@
         <item t="default"/>
       </items>
     </pivotField>
-    <pivotField showAll="0">
-      <items count="369">
+    <pivotField showAll="0" defaultSubtotal="0"/>
+    <pivotField showAll="0" defaultSubtotal="0">
+      <items count="14">
         <item x="0"/>
         <item x="1"/>
         <item x="2"/>
@@ -19945,435 +20329,66 @@
         <item x="11"/>
         <item x="12"/>
         <item x="13"/>
-        <item x="14"/>
-        <item x="15"/>
-        <item x="16"/>
-        <item x="17"/>
-        <item x="18"/>
-        <item x="19"/>
-        <item x="20"/>
-        <item x="21"/>
-        <item x="22"/>
-        <item x="23"/>
-        <item x="24"/>
-        <item x="25"/>
-        <item x="26"/>
-        <item x="27"/>
-        <item x="28"/>
-        <item x="29"/>
-        <item x="30"/>
-        <item x="31"/>
-        <item x="32"/>
-        <item x="33"/>
-        <item x="34"/>
-        <item x="35"/>
-        <item x="36"/>
-        <item x="37"/>
-        <item x="38"/>
-        <item x="39"/>
-        <item x="40"/>
-        <item x="41"/>
-        <item x="42"/>
-        <item x="43"/>
-        <item x="44"/>
-        <item x="45"/>
-        <item x="46"/>
-        <item x="47"/>
-        <item x="48"/>
-        <item x="49"/>
-        <item x="50"/>
-        <item x="51"/>
-        <item x="52"/>
-        <item x="53"/>
-        <item x="54"/>
-        <item x="55"/>
-        <item x="56"/>
-        <item x="57"/>
-        <item x="58"/>
-        <item x="59"/>
-        <item x="60"/>
-        <item x="61"/>
-        <item x="62"/>
-        <item x="63"/>
-        <item x="64"/>
-        <item x="65"/>
-        <item x="66"/>
-        <item x="67"/>
-        <item x="68"/>
-        <item x="69"/>
-        <item x="70"/>
-        <item x="71"/>
-        <item x="72"/>
-        <item x="73"/>
-        <item x="74"/>
-        <item x="75"/>
-        <item x="76"/>
-        <item x="77"/>
-        <item x="78"/>
-        <item x="79"/>
-        <item x="80"/>
-        <item x="81"/>
-        <item x="82"/>
-        <item x="83"/>
-        <item x="84"/>
-        <item x="85"/>
-        <item x="86"/>
-        <item x="87"/>
-        <item x="88"/>
-        <item x="89"/>
-        <item x="90"/>
-        <item x="91"/>
-        <item x="92"/>
-        <item x="93"/>
-        <item x="94"/>
-        <item x="95"/>
-        <item x="96"/>
-        <item x="97"/>
-        <item x="98"/>
-        <item x="99"/>
-        <item x="100"/>
-        <item x="101"/>
-        <item x="102"/>
-        <item x="103"/>
-        <item x="104"/>
-        <item x="105"/>
-        <item x="106"/>
-        <item x="107"/>
-        <item x="108"/>
-        <item x="109"/>
-        <item x="110"/>
-        <item x="111"/>
-        <item x="112"/>
-        <item x="113"/>
-        <item x="114"/>
-        <item x="115"/>
-        <item x="116"/>
-        <item x="117"/>
-        <item x="118"/>
-        <item x="119"/>
-        <item x="120"/>
-        <item x="121"/>
-        <item x="122"/>
-        <item x="123"/>
-        <item x="124"/>
-        <item x="125"/>
-        <item x="126"/>
-        <item x="127"/>
-        <item x="128"/>
-        <item x="129"/>
-        <item x="130"/>
-        <item x="131"/>
-        <item x="132"/>
-        <item x="133"/>
-        <item x="134"/>
-        <item x="135"/>
-        <item x="136"/>
-        <item x="137"/>
-        <item x="138"/>
-        <item x="139"/>
-        <item x="140"/>
-        <item x="141"/>
-        <item x="142"/>
-        <item x="143"/>
-        <item x="144"/>
-        <item x="145"/>
-        <item x="146"/>
-        <item x="147"/>
-        <item x="148"/>
-        <item x="149"/>
-        <item x="150"/>
-        <item x="151"/>
-        <item x="152"/>
-        <item x="153"/>
-        <item x="154"/>
-        <item x="155"/>
-        <item x="156"/>
-        <item x="157"/>
-        <item x="158"/>
-        <item x="159"/>
-        <item x="160"/>
-        <item x="161"/>
-        <item x="162"/>
-        <item x="163"/>
-        <item x="164"/>
-        <item x="165"/>
-        <item x="166"/>
-        <item x="167"/>
-        <item x="168"/>
-        <item x="169"/>
-        <item x="170"/>
-        <item x="171"/>
-        <item x="172"/>
-        <item x="173"/>
-        <item x="174"/>
-        <item x="175"/>
-        <item x="176"/>
-        <item x="177"/>
-        <item x="178"/>
-        <item x="179"/>
-        <item x="180"/>
-        <item x="181"/>
-        <item x="182"/>
-        <item x="183"/>
-        <item x="184"/>
-        <item x="185"/>
-        <item x="186"/>
-        <item x="187"/>
-        <item x="188"/>
-        <item x="189"/>
-        <item x="190"/>
-        <item x="191"/>
-        <item x="192"/>
-        <item x="193"/>
-        <item x="194"/>
-        <item x="195"/>
-        <item x="196"/>
-        <item x="197"/>
-        <item x="198"/>
-        <item x="199"/>
-        <item x="200"/>
-        <item x="201"/>
-        <item x="202"/>
-        <item x="203"/>
-        <item x="204"/>
-        <item x="205"/>
-        <item x="206"/>
-        <item x="207"/>
-        <item x="208"/>
-        <item x="209"/>
-        <item x="210"/>
-        <item x="211"/>
-        <item x="212"/>
-        <item x="213"/>
-        <item x="214"/>
-        <item x="215"/>
-        <item x="216"/>
-        <item x="217"/>
-        <item x="218"/>
-        <item x="219"/>
-        <item x="220"/>
-        <item x="221"/>
-        <item x="222"/>
-        <item x="223"/>
-        <item x="224"/>
-        <item x="225"/>
-        <item x="226"/>
-        <item x="227"/>
-        <item x="228"/>
-        <item x="229"/>
-        <item x="230"/>
-        <item x="231"/>
-        <item x="232"/>
-        <item x="233"/>
-        <item x="234"/>
-        <item x="235"/>
-        <item x="236"/>
-        <item x="237"/>
-        <item x="238"/>
-        <item x="239"/>
-        <item x="240"/>
-        <item x="241"/>
-        <item x="242"/>
-        <item x="243"/>
-        <item x="244"/>
-        <item x="245"/>
-        <item x="246"/>
-        <item x="247"/>
-        <item x="248"/>
-        <item x="249"/>
-        <item x="250"/>
-        <item x="251"/>
-        <item x="252"/>
-        <item x="253"/>
-        <item x="254"/>
-        <item x="255"/>
-        <item x="256"/>
-        <item x="257"/>
-        <item x="258"/>
-        <item x="259"/>
-        <item x="260"/>
-        <item x="261"/>
-        <item x="262"/>
-        <item x="263"/>
-        <item x="264"/>
-        <item x="265"/>
-        <item x="266"/>
-        <item x="267"/>
-        <item x="268"/>
-        <item x="269"/>
-        <item x="270"/>
-        <item x="271"/>
-        <item x="272"/>
-        <item x="273"/>
-        <item x="274"/>
-        <item x="275"/>
-        <item x="276"/>
-        <item x="277"/>
-        <item x="278"/>
-        <item x="279"/>
-        <item x="280"/>
-        <item x="281"/>
-        <item x="282"/>
-        <item x="283"/>
-        <item x="284"/>
-        <item x="285"/>
-        <item x="286"/>
-        <item x="287"/>
-        <item x="288"/>
-        <item x="289"/>
-        <item x="290"/>
-        <item x="291"/>
-        <item x="292"/>
-        <item x="293"/>
-        <item x="294"/>
-        <item x="295"/>
-        <item x="296"/>
-        <item x="297"/>
-        <item x="298"/>
-        <item x="299"/>
-        <item x="300"/>
-        <item x="301"/>
-        <item x="302"/>
-        <item x="303"/>
-        <item x="304"/>
-        <item x="305"/>
-        <item x="306"/>
-        <item x="307"/>
-        <item x="308"/>
-        <item x="309"/>
-        <item x="310"/>
-        <item x="311"/>
-        <item x="312"/>
-        <item x="313"/>
-        <item x="314"/>
-        <item x="315"/>
-        <item x="316"/>
-        <item x="317"/>
-        <item x="318"/>
-        <item x="319"/>
-        <item x="320"/>
-        <item x="321"/>
-        <item x="322"/>
-        <item x="323"/>
-        <item x="324"/>
-        <item x="325"/>
-        <item x="326"/>
-        <item x="327"/>
-        <item x="328"/>
-        <item x="329"/>
-        <item x="330"/>
-        <item x="331"/>
-        <item x="332"/>
-        <item x="333"/>
-        <item x="334"/>
-        <item x="335"/>
-        <item x="336"/>
-        <item x="337"/>
-        <item x="338"/>
-        <item x="339"/>
-        <item x="340"/>
-        <item x="341"/>
-        <item x="342"/>
-        <item x="343"/>
-        <item x="344"/>
-        <item x="345"/>
-        <item x="346"/>
-        <item x="347"/>
-        <item x="348"/>
-        <item x="349"/>
-        <item x="350"/>
-        <item x="351"/>
-        <item x="352"/>
-        <item x="353"/>
-        <item x="354"/>
-        <item x="355"/>
-        <item x="356"/>
-        <item x="357"/>
-        <item x="358"/>
-        <item x="359"/>
-        <item x="360"/>
-        <item x="361"/>
-        <item x="362"/>
-        <item x="363"/>
-        <item x="364"/>
-        <item x="365"/>
-        <item x="366"/>
-        <item x="367"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="15">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item x="11"/>
-        <item x="12"/>
-        <item x="13"/>
-        <item t="default"/>
       </items>
     </pivotField>
   </pivotFields>
-  <rowFields count="3">
+  <rowFields count="2">
+    <field x="0"/>
     <field x="1"/>
-    <field x="0"/>
-    <field x="5"/>
   </rowFields>
-  <rowItems count="17">
+  <rowItems count="19">
+    <i>
+      <x/>
+    </i>
+    <i r="1">
+      <x/>
+    </i>
+    <i r="1">
+      <x v="1"/>
+    </i>
+    <i r="1">
+      <x v="2"/>
+    </i>
+    <i r="1">
+      <x v="3"/>
+    </i>
+    <i r="1">
+      <x v="4"/>
+    </i>
     <i>
       <x v="1"/>
     </i>
     <i r="1">
       <x/>
     </i>
-    <i r="2">
+    <i r="1">
       <x v="1"/>
     </i>
-    <i r="2">
+    <i r="1">
       <x v="2"/>
     </i>
-    <i r="2">
+    <i r="1">
       <x v="3"/>
     </i>
-    <i r="2">
+    <i r="1">
       <x v="4"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i r="1">
+      <x/>
     </i>
     <i r="1">
       <x v="1"/>
     </i>
-    <i r="2">
-      <x v="1"/>
-    </i>
-    <i r="2">
-      <x v="2"/>
-    </i>
-    <i r="2">
-      <x v="3"/>
-    </i>
-    <i r="2">
-      <x v="4"/>
-    </i>
     <i r="1">
       <x v="2"/>
     </i>
-    <i r="2">
-      <x v="1"/>
-    </i>
-    <i r="2">
-      <x v="2"/>
-    </i>
-    <i r="2">
+    <i r="1">
       <x v="3"/>
     </i>
-    <i r="2">
+    <i r="1">
       <x v="4"/>
     </i>
     <i t="grand">
@@ -20384,10 +20399,10 @@
     <i/>
   </colItems>
   <dataFields count="1">
-    <dataField name="Sum of Price" fld="2" baseField="0" baseItem="0" numFmtId="164"/>
+    <dataField name="Max of Price" fld="2" subtotal="max" baseField="0" baseItem="0" numFmtId="164"/>
   </dataFields>
-  <chartFormats count="14">
-    <chartFormat chart="2" format="0" series="1">
+  <chartFormats count="16">
+    <chartFormat chart="3" format="12" series="1">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="1">
           <reference field="4294967294" count="1" selected="0">
@@ -20396,90 +20411,84 @@
         </references>
       </pivotArea>
     </chartFormat>
-    <chartFormat chart="4" format="2" series="1">
+    <chartFormat chart="3" format="13">
       <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
+        <references count="3">
           <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
             <x v="0"/>
           </reference>
         </references>
       </pivotArea>
     </chartFormat>
-    <chartFormat chart="4" format="3">
+    <chartFormat chart="3" format="14">
       <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="4">
+        <references count="3">
           <reference field="4294967294" count="1" selected="0">
             <x v="0"/>
           </reference>
           <reference field="0" count="1" selected="0">
-            <x v="0"/>
+            <x v="2"/>
           </reference>
           <reference field="1" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-          <reference field="5" count="1" selected="0">
             <x v="1"/>
           </reference>
         </references>
       </pivotArea>
     </chartFormat>
-    <chartFormat chart="4" format="4">
+    <chartFormat chart="3" format="15">
       <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="4">
+        <references count="3">
           <reference field="4294967294" count="1" selected="0">
             <x v="0"/>
           </reference>
           <reference field="0" count="1" selected="0">
-            <x v="0"/>
+            <x v="2"/>
           </reference>
           <reference field="1" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-          <reference field="5" count="1" selected="0">
             <x v="2"/>
           </reference>
         </references>
       </pivotArea>
     </chartFormat>
-    <chartFormat chart="4" format="5">
+    <chartFormat chart="3" format="16">
       <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="4">
+        <references count="3">
           <reference field="4294967294" count="1" selected="0">
             <x v="0"/>
           </reference>
           <reference field="0" count="1" selected="0">
-            <x v="0"/>
+            <x v="2"/>
           </reference>
           <reference field="1" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-          <reference field="5" count="1" selected="0">
             <x v="3"/>
           </reference>
         </references>
       </pivotArea>
     </chartFormat>
-    <chartFormat chart="4" format="6">
+    <chartFormat chart="3" format="17">
       <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="4">
+        <references count="3">
           <reference field="4294967294" count="1" selected="0">
             <x v="0"/>
           </reference>
           <reference field="0" count="1" selected="0">
-            <x v="0"/>
+            <x v="2"/>
           </reference>
           <reference field="1" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-          <reference field="5" count="1" selected="0">
             <x v="4"/>
           </reference>
         </references>
       </pivotArea>
     </chartFormat>
-    <chartFormat chart="4" format="7">
+    <chartFormat chart="3" format="18">
       <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="4">
+        <references count="3">
           <reference field="4294967294" count="1" selected="0">
             <x v="0"/>
           </reference>
@@ -20487,17 +20496,14 @@
             <x v="1"/>
           </reference>
           <reference field="1" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-          <reference field="5" count="1" selected="0">
-            <x v="1"/>
+            <x v="4"/>
           </reference>
         </references>
       </pivotArea>
     </chartFormat>
-    <chartFormat chart="4" format="8">
+    <chartFormat chart="3" format="19">
       <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="4">
+        <references count="3">
           <reference field="4294967294" count="1" selected="0">
             <x v="0"/>
           </reference>
@@ -20505,17 +20511,14 @@
             <x v="1"/>
           </reference>
           <reference field="1" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-          <reference field="5" count="1" selected="0">
-            <x v="2"/>
+            <x v="3"/>
           </reference>
         </references>
       </pivotArea>
     </chartFormat>
-    <chartFormat chart="4" format="9">
+    <chartFormat chart="3" format="20">
       <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="4">
+        <references count="3">
           <reference field="4294967294" count="1" selected="0">
             <x v="0"/>
           </reference>
@@ -20523,17 +20526,14 @@
             <x v="1"/>
           </reference>
           <reference field="1" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-          <reference field="5" count="1" selected="0">
-            <x v="3"/>
+            <x v="2"/>
           </reference>
         </references>
       </pivotArea>
     </chartFormat>
-    <chartFormat chart="4" format="10">
+    <chartFormat chart="3" format="21">
       <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="4">
+        <references count="3">
           <reference field="4294967294" count="1" selected="0">
             <x v="0"/>
           </reference>
@@ -20541,82 +20541,97 @@
             <x v="1"/>
           </reference>
           <reference field="1" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-          <reference field="5" count="1" selected="0">
-            <x v="4"/>
+            <x v="0"/>
           </reference>
         </references>
       </pivotArea>
     </chartFormat>
-    <chartFormat chart="4" format="11">
+    <chartFormat chart="3" format="22">
       <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="4">
+        <references count="3">
           <reference field="4294967294" count="1" selected="0">
             <x v="0"/>
           </reference>
           <reference field="0" count="1" selected="0">
-            <x v="2"/>
+            <x v="1"/>
           </reference>
           <reference field="1" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-          <reference field="5" count="1" selected="0">
             <x v="1"/>
           </reference>
         </references>
       </pivotArea>
     </chartFormat>
-    <chartFormat chart="4" format="12">
+    <chartFormat chart="3" format="23">
       <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="4">
+        <references count="3">
           <reference field="4294967294" count="1" selected="0">
             <x v="0"/>
           </reference>
           <reference field="0" count="1" selected="0">
-            <x v="2"/>
+            <x v="0"/>
           </reference>
           <reference field="1" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-          <reference field="5" count="1" selected="0">
             <x v="2"/>
           </reference>
         </references>
       </pivotArea>
     </chartFormat>
-    <chartFormat chart="4" format="13">
+    <chartFormat chart="3" format="24">
       <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="4">
+        <references count="3">
           <reference field="4294967294" count="1" selected="0">
             <x v="0"/>
           </reference>
           <reference field="0" count="1" selected="0">
-            <x v="2"/>
+            <x v="0"/>
           </reference>
           <reference field="1" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-          <reference field="5" count="1" selected="0">
-            <x v="3"/>
+            <x v="4"/>
           </reference>
         </references>
       </pivotArea>
     </chartFormat>
-    <chartFormat chart="4" format="14">
+    <chartFormat chart="3" format="25">
       <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="4">
+        <references count="3">
           <reference field="4294967294" count="1" selected="0">
             <x v="0"/>
           </reference>
           <reference field="0" count="1" selected="0">
-            <x v="2"/>
+            <x v="0"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="3" format="26">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="3">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="1" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="3" format="27">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="3">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="0" count="1" selected="0">
+            <x v="0"/>
           </reference>
           <reference field="1" count="1" selected="0">
             <x v="1"/>
-          </reference>
-          <reference field="5" count="1" selected="0">
-            <x v="4"/>
           </reference>
         </references>
       </pivotArea>

</xml_diff>